<commit_message>
add picturies in price.xlsx
</commit_message>
<xml_diff>
--- a/files/management/commands/price.xlsx
+++ b/files/management/commands/price.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="delivery" sheetId="1" state="visible" r:id="rId3"/>
@@ -17,6 +17,7 @@
     <sheet name="blank_material" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="interierka" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="finishka" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="picturies" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="85">
   <si>
     <t xml:space="preserve">№</t>
   </si>
@@ -216,7 +217,7 @@
     <t xml:space="preserve">Пленка ПЭТ Беклит 215 гр (1,24 м)</t>
   </si>
   <si>
-    <t xml:space="preserve">Холст искуственный Мат; Гл. 260 гр </t>
+    <t xml:space="preserve">Холст искусственный Мат; Гл. 260 гр </t>
   </si>
   <si>
     <t xml:space="preserve">Фотообои </t>
@@ -247,6 +248,42 @@
   </si>
   <si>
     <t xml:space="preserve">Без полей</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Картина Холст на подрамнике 20х30 см </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Картина Холст на подрамнике 30х30 см </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Картина Холст на подрамнике 30х40 см </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Картина Холст на подрамнике 40х40 см </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Картина Холст на подрамнике 40х50 см </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Картина Холст на подрамнике 40х60 см </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Картина Холст на подрамнике 50х50 см </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Картина Холст на подрамнике 50х70 см </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Картина Холст на подрамнике 60х60 см </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Картина Холст на подрамнике 60х70 см </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Картина Холст на подрамнике 60х90 см </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Картина Холст на подрамнике 90х120 см </t>
   </si>
 </sst>
 </file>
@@ -746,6 +783,322 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="61.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="21.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="27.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="29.67"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4"/>
+      <c r="B1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>750</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>1750</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>1875</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>1050</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>2050</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>2050</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>1150</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>2150</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>2150</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>230</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>2350</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>2350</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>280</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>2400</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>2400</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>490</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>490</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>2900</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>2900</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>550</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>2900</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>2900</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>345</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>3150</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>3150</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>450</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>3300</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>3300</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>670</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>

<commit_message>
edit price.xlsx - 3
</commit_message>
<xml_diff>
--- a/files/management/commands/price.xlsx
+++ b/files/management/commands/price.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="delivery" sheetId="1" state="visible" r:id="rId3"/>
@@ -850,7 +850,6 @@
         <v>2050</v>
       </c>
       <c r="E3" s="7" t="n">
-        <f aca="false">C3*2.5</f>
         <v>2625</v>
       </c>
       <c r="F3" s="7" t="n">
@@ -2770,7 +2769,6 @@
         <v>520</v>
       </c>
       <c r="E2" s="7" t="n">
-        <f aca="false">C2*2.5</f>
         <v>725</v>
       </c>
       <c r="F2" s="7" t="n">

</xml_diff>

<commit_message>
add Interest in execel
</commit_message>
<xml_diff>
--- a/files/management/commands/price.xlsx
+++ b/files/management/commands/price.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="11"/>
   </bookViews>
   <sheets>
     <sheet name="delivery" sheetId="1" state="visible" r:id="rId3"/>
@@ -18,6 +18,8 @@
     <sheet name="interierka" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="finishka" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="picturies" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="lid_interes" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="lid_status" sheetId="12" state="visible" r:id="rId14"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="102">
   <si>
     <t xml:space="preserve">№</t>
   </si>
@@ -287,6 +289,54 @@
   </si>
   <si>
     <t xml:space="preserve">Картина Холст на подрамнике 90х120 см </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Печать баннера </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Изготовление таблички</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Лазерная резка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Стенды</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пресс волы</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ролл апы</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Планы Эвакуации</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Печать на холсте</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ответил на вопросы</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выслал дополнительную информацию</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выставил счет</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Разработка макета</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В производстве</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Заказ Готов</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сообщение о доставке</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Просим отзыв о работе</t>
   </si>
 </sst>
 </file>
@@ -407,7 +457,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -466,10 +516,6 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1106,6 +1152,206 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44.56"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4"/>
+      <c r="B1" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.92"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4"/>
+      <c r="B1" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -3329,19 +3575,19 @@
       <c r="L8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="7" t="n">
         <v>100</v>
       </c>
       <c r="F9" s="6"/>

</xml_diff>

<commit_message>
edit temlpate lid list detail list
</commit_message>
<xml_diff>
--- a/files/management/commands/price.xlsx
+++ b/files/management/commands/price.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="delivery" sheetId="1" state="visible" r:id="rId3"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="92">
   <si>
     <t xml:space="preserve">№</t>
   </si>
@@ -1082,7 +1082,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1139,6 +1139,14 @@
       </c>
       <c r="B7" s="3" t="s">
         <v>91</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add position in price.xlsx
</commit_message>
<xml_diff>
--- a/files/management/commands/price.xlsx
+++ b/files/management/commands/price.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="delivery" sheetId="1" state="visible" r:id="rId3"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="93">
   <si>
     <t xml:space="preserve">№</t>
   </si>
@@ -249,6 +249,9 @@
   </si>
   <si>
     <t xml:space="preserve">Без полей</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Проварка края</t>
   </si>
   <si>
     <t xml:space="preserve">Картина Холст на подрамнике 20х30 см </t>
@@ -740,7 +743,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.57"/>
@@ -811,7 +814,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="61.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.31"/>
@@ -839,7 +842,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C2" s="7" t="n">
         <v>750</v>
@@ -856,7 +859,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>1050</v>
@@ -873,7 +876,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C4" s="7" t="n">
         <v>1150</v>
@@ -890,7 +893,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C5" s="7" t="n">
         <v>230</v>
@@ -907,7 +910,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>280</v>
@@ -924,7 +927,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>420</v>
@@ -941,7 +944,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>490</v>
@@ -958,7 +961,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>490</v>
@@ -975,7 +978,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>550</v>
@@ -992,7 +995,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C11" s="7" t="n">
         <v>345</v>
@@ -1009,7 +1012,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C12" s="7" t="n">
         <v>450</v>
@@ -1026,7 +1029,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>670</v>
@@ -1083,14 +1086,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1098,7 +1101,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1106,7 +1109,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1114,7 +1117,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1122,7 +1125,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1130,7 +1133,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1138,15 +1141,15 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>91</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="0" t="s">
-        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1166,7 +1169,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.57"/>
@@ -1245,7 +1248,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="58.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.57"/>
@@ -1582,7 +1585,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.42"/>
   </cols>
@@ -1644,7 +1647,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
@@ -1695,7 +1698,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G69"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="13.45" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="13.45" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="56.57"/>
@@ -2452,7 +2455,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F14"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="58.42"/>
@@ -2639,7 +2642,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="61.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.57"/>
@@ -2986,7 +2989,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L43"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="13.45" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="13.45" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="57.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.29"/>
@@ -3227,11 +3230,21 @@
       <c r="L10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="13.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>69</v>
+      </c>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>

</xml_diff>

<commit_message>
add price.xlsx position inrtrier pirnt Matte and Glossy Films
</commit_message>
<xml_diff>
--- a/files/management/commands/price.xlsx
+++ b/files/management/commands/price.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="delivery" sheetId="1" state="visible" r:id="rId3"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="95">
   <si>
     <t xml:space="preserve">№</t>
   </si>
@@ -206,7 +206,13 @@
     <t xml:space="preserve">Пленка Евро Мат;Гл.;Пр.  80 гр (1,05; 1,27; 1,37; 1,52 м)</t>
   </si>
   <si>
-    <t xml:space="preserve">Пленка Китай Мат;Гл.;Пр.  100 гр (1,05; 1,27; 1,37; 1,52 м)</t>
+    <t xml:space="preserve">Пленка Китай Матовая 100 гр</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пленка Китай Глянцевая 100 гр</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пленка Китай Прозрачная 100 гр</t>
   </si>
   <si>
     <t xml:space="preserve">Пленка перфорированная (черный оборот) 140 гр (1,37 м)</t>
@@ -842,7 +848,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C2" s="7" t="n">
         <v>750</v>
@@ -859,7 +865,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>1050</v>
@@ -876,7 +882,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C4" s="7" t="n">
         <v>1150</v>
@@ -893,7 +899,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C5" s="7" t="n">
         <v>230</v>
@@ -910,7 +916,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>280</v>
@@ -927,7 +933,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>420</v>
@@ -944,7 +950,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>490</v>
@@ -961,7 +967,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>490</v>
@@ -978,7 +984,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>550</v>
@@ -995,7 +1001,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C11" s="7" t="n">
         <v>345</v>
@@ -1012,7 +1018,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C12" s="7" t="n">
         <v>450</v>
@@ -1029,7 +1035,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>670</v>
@@ -1093,7 +1099,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1101,7 +1107,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1109,7 +1115,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1117,7 +1123,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1125,7 +1131,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1133,7 +1139,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1141,7 +1147,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1149,7 +1155,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -2641,7 +2647,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.45" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="61.95"/>
@@ -2844,13 +2850,13 @@
         <v>59</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>450</v>
+        <v>345</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>765</v>
+        <v>460</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>1125</v>
+        <v>865</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2861,13 +2867,13 @@
         <v>60</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>670</v>
+        <v>345</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>1140</v>
+        <v>460</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>1675</v>
+        <v>865</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2875,74 +2881,102 @@
         <v>13</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>28</v>
+        <v>61</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>730</v>
+        <v>450</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>1200</v>
+        <v>765</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>1825</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="14" t="s">
-        <v>61</v>
+      <c r="B15" s="6" t="s">
+        <v>62</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>590</v>
+        <v>670</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>1060</v>
+        <v>1140</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>1475</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="14" t="s">
-        <v>62</v>
+      <c r="B16" s="6" t="s">
+        <v>28</v>
       </c>
       <c r="C16" s="7" t="n">
+        <v>730</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>1825</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>590</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>1060</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" s="7" t="n">
         <v>550</v>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D18" s="7" t="n">
         <v>900</v>
       </c>
-      <c r="E16" s="7" t="n">
+      <c r="E18" s="7" t="n">
         <v>1375</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C17" s="7" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" s="7" t="n">
         <v>520</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D19" s="7" t="n">
         <v>1100</v>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="E19" s="7" t="n">
         <v>1300</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6"/>
@@ -2955,22 +2989,28 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6"/>
-      <c r="B23" s="6"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6"/>
-      <c r="B24" s="6"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
       <c r="C25" s="7"/>
       <c r="D25" s="7"/>
       <c r="E25" s="7"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3024,7 +3064,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C2" s="7" t="n">
         <v>0</v>
@@ -3047,7 +3087,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>10</v>
@@ -3070,7 +3110,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C4" s="7" t="n">
         <v>60</v>
@@ -3093,7 +3133,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C5" s="7" t="n">
         <v>80</v>
@@ -3116,7 +3156,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>100</v>
@@ -3139,7 +3179,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>100</v>
@@ -3162,7 +3202,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>100</v>
@@ -3186,7 +3226,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>60</v>
@@ -3210,7 +3250,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C10" s="7" t="n">
         <v>0</v>
@@ -3229,12 +3269,12 @@
       <c r="K10" s="6"/>
       <c r="L10" s="6"/>
     </row>
-    <row r="11" customFormat="false" ht="13.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>30</v>

</xml_diff>